<commit_message>
Final changes has made
</commit_message>
<xml_diff>
--- a/MegaProject/Automated Test Execution/data/bcm_testcases.xlsx
+++ b/MegaProject/Automated Test Execution/data/bcm_testcases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://weedag-my.sharepoint.com/personal/omkar_hande_edag_com/Documents/Raw_project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oh99312\Desktop\Updated\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="11_325F69DB08E94A1694601FB188D7A06D41A21DC4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8972AE65-F691-4F62-A156-E5FE85954CDD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A97C12-1C45-4C82-A231-05B659AC0B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="47">
   <si>
     <t>TC_ID</t>
   </si>
@@ -31,9 +31,6 @@
     <t>Ignition_ON/OFF</t>
   </si>
   <si>
-    <t>Vehicle_Speed_ (km/h)</t>
-  </si>
-  <si>
     <t>Driver_Door</t>
   </si>
   <si>
@@ -58,9 +55,6 @@
     <t>TC01</t>
   </si>
   <si>
-    <t>Lock door using key fob</t>
-  </si>
-  <si>
     <t>OFF</t>
   </si>
   <si>
@@ -79,9 +73,6 @@
     <t>TC02</t>
   </si>
   <si>
-    <t>Unlock door using key fob</t>
-  </si>
-  <si>
     <t>unlock_keyfob</t>
   </si>
   <si>
@@ -103,15 +94,9 @@
     <t>TC05</t>
   </si>
   <si>
-    <t>Verify unlock at boundary value 60 km/h</t>
-  </si>
-  <si>
     <t>TC06</t>
   </si>
   <si>
-    <t>Verify auto-lock activates above 20 km/h</t>
-  </si>
-  <si>
     <t>auto_lock</t>
   </si>
   <si>
@@ -121,37 +106,61 @@
     <t>TC08</t>
   </si>
   <si>
-    <t>Verify lock command when driver door is open</t>
-  </si>
-  <si>
     <t>TC09</t>
   </si>
   <si>
-    <t>Verify central lock request</t>
-  </si>
-  <si>
     <t>central_lock</t>
   </si>
   <si>
     <t>TC10</t>
   </si>
   <si>
-    <t>Verify central unlock request</t>
-  </si>
-  <si>
     <t>TC11</t>
   </si>
   <si>
-    <t>Verify lock request when boot door open</t>
-  </si>
-  <si>
-    <t>Verify unlock is allowed at low speed value&lt;10</t>
-  </si>
-  <si>
-    <t>Verify unlock is blocked above speed limit&gt;10</t>
-  </si>
-  <si>
-    <t>Verify auto-lock does not activate below threshold(20)</t>
+    <t>TC12</t>
+  </si>
+  <si>
+    <t>Vehicle_Speed_(km/h)</t>
+  </si>
+  <si>
+    <t>Verify that all vehicle doors are locked successfully when the Lock button on the key fob is pressed</t>
+  </si>
+  <si>
+    <t>Verify that all vehicle doors are unlocked successfully when the Unlock button on the key fob is pressed </t>
+  </si>
+  <si>
+    <t>Verify that door unlock operation is allowed using the central unlocking switch when vehicle speed is below 10 km/h</t>
+  </si>
+  <si>
+    <t>Verify that door unlock operation is blocked using the central unlocking switch when vehicle speed exceeds 10 km/h </t>
+  </si>
+  <si>
+    <t>Verify that automatic door locking is activated when vehicle speed exceeds 20 km/h</t>
+  </si>
+  <si>
+    <t>Verify that key fob lock request is rejected when the driver door is open</t>
+  </si>
+  <si>
+    <t>Verify that all vehicle doors are locked successfully using the central locking switch</t>
+  </si>
+  <si>
+    <t>Verify that all vehicle doors are unlocked successfully using the central unlocking switch</t>
+  </si>
+  <si>
+    <t>Verify that lock request through the key fob is rejected when the boot door is open and the vehicle is parked </t>
+  </si>
+  <si>
+    <t>closed</t>
+  </si>
+  <si>
+    <t>TC13</t>
+  </si>
+  <si>
+    <t>Verify lock request when some fields are missing</t>
+  </si>
+  <si>
+    <t>Verify that central unlock request is allowed or not at the vehicle speed of 60 km/h </t>
   </si>
 </sst>
 </file>
@@ -529,10 +538,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.69921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.69921875" customWidth="1"/>
+    <col min="2" max="2" width="100.69921875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.8984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.296875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
@@ -544,7 +553,7 @@
     <col min="11" max="11" width="14.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -555,422 +564,515 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
         <v>11</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" t="s">
-        <v>13</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="K2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" t="s">
         <v>15</v>
       </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4">
         <v>30</v>
       </c>
       <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" t="s">
         <v>15</v>
       </c>
-      <c r="F4" t="s">
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6">
+        <v>60</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7">
         <v>15</v>
       </c>
-      <c r="G4" t="s">
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" t="s">
+        <v>25</v>
+      </c>
+      <c r="K7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" t="s">
+        <v>25</v>
+      </c>
+      <c r="K8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9">
         <v>15</v>
       </c>
-      <c r="H4" t="s">
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" t="s">
         <v>15</v>
       </c>
-      <c r="I4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5">
-        <v>70</v>
-      </c>
-      <c r="E5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" t="s">
-        <v>15</v>
-      </c>
-      <c r="J5" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>27</v>
       </c>
-      <c r="C6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6">
-        <v>50</v>
-      </c>
-      <c r="E6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" t="s">
-        <v>23</v>
-      </c>
-      <c r="K6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" t="s">
-        <v>15</v>
-      </c>
-      <c r="J7" t="s">
-        <v>30</v>
-      </c>
-      <c r="K7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8">
-        <v>15</v>
-      </c>
-      <c r="E8" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" t="s">
-        <v>15</v>
-      </c>
-      <c r="J8" t="s">
-        <v>30</v>
-      </c>
-      <c r="K8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I9" t="s">
-        <v>15</v>
-      </c>
-      <c r="J9" t="s">
-        <v>16</v>
-      </c>
-      <c r="K9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>34</v>
-      </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J10" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="K10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" t="s">
+        <v>13</v>
+      </c>
+      <c r="J11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K11" t="s">
         <v>15</v>
       </c>
-      <c r="F11" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" t="s">
-        <v>15</v>
-      </c>
-      <c r="I11" t="s">
-        <v>15</v>
-      </c>
-      <c r="J11" t="s">
-        <v>23</v>
-      </c>
-      <c r="K11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I12" t="s">
+        <v>12</v>
+      </c>
+      <c r="J12" t="s">
+        <v>14</v>
+      </c>
+      <c r="K12" t="s">
         <v>15</v>
       </c>
-      <c r="F12" t="s">
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" t="s">
+        <v>13</v>
+      </c>
+      <c r="J13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" t="s">
+        <v>43</v>
+      </c>
+      <c r="H14" t="s">
+        <v>13</v>
+      </c>
+      <c r="I14" t="s">
+        <v>43</v>
+      </c>
+      <c r="J14" t="s">
+        <v>14</v>
+      </c>
+      <c r="K14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" t="s">
+        <v>13</v>
+      </c>
+      <c r="I15" t="s">
+        <v>13</v>
+      </c>
+      <c r="J15" t="s">
+        <v>17</v>
+      </c>
+      <c r="K15" t="s">
         <v>15</v>
       </c>
-      <c r="G12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" t="s">
-        <v>15</v>
-      </c>
-      <c r="I12" t="s">
-        <v>14</v>
-      </c>
-      <c r="J12" t="s">
-        <v>16</v>
-      </c>
-      <c r="K12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:K1 A7:K7 A5 A6:C6 A16:K23 A10:B10 A11:J11 A3:K3 A2:J2 A4 C4 E4:K4 C5:G5 I5:J5 E6:J6 A9:K9 A8 C8:K8 D10:J10" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C1 A8 A5 A6 A16:K20 A11 A12 A3 A2 A4 C4 E4:K4 C5 I5:J5 E6:J6 A10 A9 C9:D9 D11:I11 E5:G5 E1:K1 C2:J2 C3:K3 C6 C8:E8 C10:I10 C12:H12 A22:K23 A21:G21 I21:K21 F9:G9 I9 K8 K9 G8:I8" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>